<commit_message>
Changes made for cord inspect module and sanity for steel cord
</commit_message>
<xml_diff>
--- a/src/main/resources/excel_data/ConveyorBulkUpload1.xlsx
+++ b/src/main/resources/excel_data/ConveyorBulkUpload1.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="26731"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27328"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Vishmitha G\Downloads\ctp-contiplus-web-qa-automation-java\ctp-contiplus-web-qa-automation-java\src\main\resources\excel_data\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Vishmitha G\Documents\Automation\ctp-contiplus-web-qa-automation-java\src\main\resources\excel_data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8030C219-FFEC-4FA3-8A43-F63A45A423ED}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1978C57C-A91F-4223-8184-EF67F9D4E20C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -250,7 +250,7 @@
     <t>Mechanical</t>
   </si>
   <si>
-    <t>BulkImport01</t>
+    <t>BulkImport1</t>
   </si>
 </sst>
 </file>

</xml_diff>

<commit_message>
fixes done during regression cycle
</commit_message>
<xml_diff>
--- a/src/main/resources/excel_data/ConveyorBulkUpload1.xlsx
+++ b/src/main/resources/excel_data/ConveyorBulkUpload1.xlsx
@@ -1,19 +1,19 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27328"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10211"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Vishmitha G\Documents\Automation\ctp-contiplus-web-qa-automation-java\src\main\resources\excel_data\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/ostan/Documents/Automation/ctp-contiplus-web-qa-automation-java_ostan/ctp-contiplus-web-qa-automation-java/src/main/resources/excel_data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1978C57C-A91F-4223-8184-EF67F9D4E20C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4370BA05-7AF2-6C4F-89BE-02B0CCCFA1AD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="760" windowWidth="23260" windowHeight="12460" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="Master" sheetId="1" r:id="rId1"/>
+    <sheet name="Cust Automation Sanity Site Aus" sheetId="1" r:id="rId1"/>
   </sheets>
   <calcPr calcId="0"/>
 </workbook>
@@ -323,9 +323,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 - 2022 Theme">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2013 - 2022">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -363,7 +363,7 @@
         <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2013 - 2022">
       <a:majorFont>
         <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
@@ -469,7 +469,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2013 - 2022">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -611,7 +611,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office 2013 - 2022 Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -620,15 +620,15 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:AH3"/>
-  <sheetFormatPr defaultColWidth="11.19921875" defaultRowHeight="15.6" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="11.1640625" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="2" max="2" width="26" customWidth="1"/>
-    <col min="3" max="3" width="19.19921875" customWidth="1"/>
+    <col min="3" max="3" width="19.1640625" customWidth="1"/>
     <col min="4" max="4" width="17.5" customWidth="1"/>
-    <col min="5" max="5" width="19.796875" customWidth="1"/>
+    <col min="5" max="5" width="19.83203125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:34" ht="43.2" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:34" ht="48" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -732,7 +732,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="2" spans="1:34" ht="46.8" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:34" ht="68" x14ac:dyDescent="0.2">
       <c r="A2" s="2" t="s">
         <v>34</v>
       </c>
@@ -836,7 +836,7 @@
         <v>63</v>
       </c>
     </row>
-    <row r="3" spans="1:34" ht="46.8" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:34" ht="68" x14ac:dyDescent="0.2">
       <c r="A3" s="2" t="s">
         <v>76</v>
       </c>

</xml_diff>